<commit_message>
Updated Program Output KPI and Service unit KPIs
</commit_message>
<xml_diff>
--- a/data/Service Unit KPIs.xlsx
+++ b/data/Service Unit KPIs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Learning\Miscellaneous\KPIDashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3959592A-E29F-4060-A714-A62C4DF07E4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41FBC3E5-94EE-4F96-A5B5-B589A46BAEF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B2484485-475C-4522-9B1B-61000E3901F6}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{B2484485-475C-4522-9B1B-61000E3901F6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="43">
   <si>
     <t>Number of datasets submitted</t>
   </si>
@@ -162,6 +162,9 @@
   </si>
   <si>
     <t>KPI Metric</t>
+  </si>
+  <si>
+    <t>In Progress</t>
   </si>
 </sst>
 </file>
@@ -17868,7 +17871,9 @@
       <c r="A23" s="44" t="s">
         <v>23</v>
       </c>
-      <c r="B23" s="47"/>
+      <c r="B23" s="47" t="s">
+        <v>42</v>
+      </c>
       <c r="C23" s="47"/>
       <c r="D23" s="56"/>
     </row>
@@ -17981,7 +17986,9 @@
       <c r="A32" s="44" t="s">
         <v>35</v>
       </c>
-      <c r="B32" s="47"/>
+      <c r="B32" s="47" t="s">
+        <v>42</v>
+      </c>
       <c r="C32" s="47"/>
       <c r="D32" s="56"/>
     </row>

</xml_diff>